<commit_message>
Traktandenliste der nächsten Sitzung aktualisieren
</commit_message>
<xml_diff>
--- a/data/traktandenliste.xlsx
+++ b/data/traktandenliste.xlsx
@@ -236,18 +236,19 @@
           <t xml:space="preserve">5</t>
         </is>
       </c>
-      <c r="B6" s="0"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026.27</t>
+        </is>
+      </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download</t>
+          <t xml:space="preserve">Verordnung / Rechtserlass</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einführung einer zentralen Digitalisierungslösung für den physischen Posteingang: Neuerlass einer Verordnung über die zentrale interne Briefpostzustellung
-2026.27W (PDF, 93 kB)
-Dokumentdatum:
-Kategorie: Antrag Stadtrat</t>
+          <t xml:space="preserve">Einführung einer zentralen Digitalisierungslösung für den physischen Posteingang: Neuerlass einer Verordnung über die zentrale interne Briefpostzustellung</t>
         </is>
       </c>
       <c r="E6" s="0"/>
@@ -259,16 +260,22 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026.27W - Beilage 1: Verordnung über die zentrale interne Briefpostzustellung Arbeitsversion (PDF, 275 kB)
-Dokumentdatum:
-Kategorie: Beilage</t>
-        </is>
-      </c>
-      <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026.62</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kreditantrag</t>
+        </is>
+      </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download</t>
+          <t xml:space="preserve">Liegenschaft Stadthausstrasse 8, «Bühne am Stadtgarten», Arealöffnung und Fassadensanierung (Projekt-Nr. 5021380): Nachtragskredit von Fr. 300'000 (vorbehältlich der Beschlussfassung in der Aufsichtskommission)</t>
         </is>
       </c>
       <c r="E7" s="0"/>
@@ -280,16 +287,22 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026.27W - Beilage 2: Verordnung über die zentrale interne Briefpostzustellung Entwurf mit Kommentar (PDF, 142 kB)
-Dokumentdatum:
-Kategorie: Beilage</t>
-        </is>
-      </c>
-      <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.29</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motion</t>
+        </is>
+      </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download</t>
+          <t xml:space="preserve">Antrag und Bericht zur Motion betr. Berücksichtigung des Wohnsitzes bei Eintrittspreisen für Sport &amp; Kultur (vorbehältlich der Beschlussfassung in der Aufsichtskommission)</t>
         </is>
       </c>
       <c r="E8" s="0"/>
@@ -301,16 +314,22 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026.27W - Beilage 3: Entwurf Vollzugsverordnung über die zentrale interne Briefpostzustellung Entwurf mit Kommentar (PDF, 195 kB)
-Dokumentdatum:
-Kategorie: Beilage</t>
-        </is>
-      </c>
-      <c r="B9" s="0"/>
-      <c r="C9" s="0"/>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026.67</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motion</t>
+        </is>
+      </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download</t>
+          <t xml:space="preserve">Begründung der Motion betr. Wahltermine für Parlaments- und Stadtratswahlen</t>
         </is>
       </c>
       <c r="E9" s="0"/>
@@ -322,16 +341,22 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026.27W - inkl. Beilagen (PDF, 566 kB)
-Dokumentdatum:
-Kategorie: Antrag Stadtrat</t>
-        </is>
-      </c>
-      <c r="B10" s="0"/>
-      <c r="C10" s="0"/>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026.87</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fragestunde</t>
+        </is>
+      </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download</t>
+          <t xml:space="preserve">Fragestunde vom 14. September 2026 (Beginn 20.00 Uhr am 14.9.2026)</t>
         </is>
       </c>
       <c r="E10" s="0"/>
@@ -340,12 +365,269 @@
       <c r="H10" s="0"/>
       <c r="I10" s="0"/>
     </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026.56</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kreditantrag</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verpflichtungskredit von Fr. 4'000'000 als Standortbeitrag zugunsten der Stiftung Technorama für die Sanierung des Gebäudes und Weiterentwicklung des Swiss Science Center Technorama (Projekt Nr. 5019670) (Behandlung am 28.9.2026 vorbehältlich der Beschlussfassung in der Sachkommission am 21.9.2026)</t>
+        </is>
+      </c>
+      <c r="E11" s="0"/>
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.101</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Postulat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Antrag und Bericht zum Postulat betr. Verbesserung des digitalen Zugangs zu amtlichen Publikationen und Stadtratsbeschlüssen (Behandlung am 28.9.2026 vorbehältlich der Beschlussfassung in der Aufsichtskommission am 21.9.2026)</t>
+        </is>
+      </c>
+      <c r="E12" s="0"/>
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.46</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. Digitalisierung von Dolmetschenden Diensten in der städtischen Verwaltung</t>
+        </is>
+      </c>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.66</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. Arbeitsplatzquote Lessons Learned</t>
+        </is>
+      </c>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.82</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. Winterthur als Migrationsstadt</t>
+        </is>
+      </c>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.121</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. «Lädelisterben» in der Altstadt Winterthur</t>
+        </is>
+      </c>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.28</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Postulat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Antrag und Bericht zum Postulat betr. private Mandatspersonen (PriMa) zur Führung von Beistandschaften</t>
+        </is>
+      </c>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.67</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. Weiterbildung und Sensibilisierung bei Radikalisierung und gewalttätigem Extremismus</t>
+        </is>
+      </c>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025.100</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interpellation</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beantwortung der Interpellation betr. Zusammensetzung überdepartementaler Gremien und institutionelle Vernetzung der Kinder- und Erwachsenenschutzbehörde (KESB) Winterthur-Andelfingen in städtischen Gremien</t>
+        </is>
+      </c>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I19"/>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rHl1"/>
     <hyperlink ref="B4" r:id="rHl2"/>
     <hyperlink ref="B5" r:id="rHl3"/>
+    <hyperlink ref="B6" r:id="rHl4"/>
+    <hyperlink ref="B7" r:id="rHl5"/>
+    <hyperlink ref="B8" r:id="rHl6"/>
+    <hyperlink ref="B9" r:id="rHl7"/>
+    <hyperlink ref="B10" r:id="rHl8"/>
+    <hyperlink ref="B11" r:id="rHl9"/>
+    <hyperlink ref="B12" r:id="rHl10"/>
+    <hyperlink ref="B13" r:id="rHl11"/>
+    <hyperlink ref="B14" r:id="rHl12"/>
+    <hyperlink ref="B15" r:id="rHl13"/>
+    <hyperlink ref="B16" r:id="rHl14"/>
+    <hyperlink ref="B17" r:id="rHl15"/>
+    <hyperlink ref="B18" r:id="rHl16"/>
+    <hyperlink ref="B19" r:id="rHl17"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>